<commit_message>
fix: harden keyword discovery pilot boundaries
</commit_message>
<xml_diff>
--- a/inputs/keyword_discovery_queries.example.xlsx
+++ b/inputs/keyword_discovery_queries.example.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검색작업" sheetId="1" r:id="R45d0255769dc4f72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검색작업" sheetId="1" r:id="Rf3013252b01e4b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자사매장" sheetId="2" r:id="Rd4cd14d27f1147c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -391,4 +392,47 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>매장ID</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="str">
+        <x:v>매장명</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="str">
+        <x:v>네이버플레이스ID</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>수동매핑플레이스ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>SAMPLE-S1</x:v>
+      </x:c>
+      <x:c r="B2" s="8" t="str">
+        <x:v>예시 매장</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="str">
+        <x:v>1001</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>legacy-1001</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>